<commit_message>
feat(users): accepte Collaborateur/Manager et Masculin/Féminin dans l'import Kostango
- Rôle : "Collaborateur" -> employee, "Manager" -> manager (les valeurs
  internes existantes restent acceptées en repli)
- Sexe : "Masculin"/"Féminin" ajoutés en plus de "Homme"/"Femme"
- templates et exemple xlsx mis à jour en conséquence
</commit_message>
<xml_diff>
--- a/doc/template_utilisateurs_kostango_exemple.xlsx
+++ b/doc/template_utilisateurs_kostango_exemple.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Homme / Femme, laisser vide sinon (optionnel)</t>
+          <t>Masculin / Féminin, laisser vide sinon (optionnel)</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>Rôle applicatif : admin / rh / manager / employee / stagiaire / alternant (employee par défaut)</t>
+          <t>Rôle applicatif : Collaborateur / Manager (Collaborateur par défaut)</t>
         </is>
       </c>
       <c r="P5" s="4" t="inlineStr">
@@ -687,7 +687,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Homme</t>
+          <t>Masculin</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>employee</t>
+          <t>Collaborateur</t>
         </is>
       </c>
       <c r="P6" t="inlineStr"/>
@@ -762,7 +762,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Femme</t>
+          <t>Féminin</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>rh</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>

</xml_diff>